<commit_message>
Fix registry cells: Sensitivity -> workbook-owned, Event Type -> code-owned (puddlejumper source)
The workbook D/E/H metadata cells for the two reclassified rows; the prior
commit carried the validator logic + findings doc. Sensitivity D21/H21 stop
claiming a source it never had; Event Type D15/E15/H15 name the real code
source in puddlejumper.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAv7tVCy2hbSMpZ9X88jpW
</commit_message>
<xml_diff>
--- a/publiclogic/canon/PublicLogic_PuddleJumper_Runtime.xlsx
+++ b/publiclogic/canon/PublicLogic_PuddleJumper_Runtime.xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canon Registry" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canon Collisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Vocabulary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Envelope" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifact Registry" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PJ Event Log" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signal Intake" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Queue" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumers" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Overview" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intake" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Steps" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Architecture" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Canon Registry" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Canon Collisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Control" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Taxonomy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Event Vocabulary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Event Envelope" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Artifact Registry" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="PJ Event Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Signal Intake" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Review Queue" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Sources" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Consumers" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Validation" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Case Overview" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Intake" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Documents" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Decisions" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Next Steps" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="LaneList">Control!$B$14:$B$17</definedName>
@@ -11706,12 +11706,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>This workbook</t>
+          <t>puddlejumper/apps/puddlejumper/src/archieve/event-catalog.ts</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Event Vocabulary sheet</t>
+          <t>ArchieveEventType</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -11723,7 +11723,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Workbook</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LogicOS Build Spec v3 (SQLite CHECK)</t>
+          <t>This workbook (governance vocabulary; no runtime enforces it)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Workbook</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">

</xml_diff>